<commit_message>
Reorganiza notebooks por fonte e cria Silver de reclamacoes
- Notebooks separados em base/, continuity/ e complaints/, com numeracao
  reiniciada; docs/img espelha a mesma estrutura
- Localizacao da raiz do repositorio por busca ascendente da pasta src,
  para funcionar em qualquer profundidade
- data/reference/reh_2992_tipologia.csv: transcricao do Anexo I da
  REH 2.992/2021 (132 codigos)
- complaints/01_silver_reference: dim_tipologia (recortes item 285 e
  comercial estrito) e dim_tempo (jan/2024 a jun/2026)
- complaints/02_silver_complaints: fato_manifestacao e
  controle_anomalias_manifestacao, com remocao de copias exatas,
  exclusao de codigos fora da REH, deteccao de meses anomalos por bloco
  e imputacao no comercial estrito do nivel 1
- screenshots.xlsx/md atualizados com os novos caminhos e a evidencia
  de validacao da ANEEL
- sessions.md com as decisoes de 23 e 24/09
</commit_message>
<xml_diff>
--- a/docs/screenshots.xlsx
+++ b/docs/screenshots.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -427,42 +439,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>arquivo_destino</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>pasta_destino</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>secao_readme</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>origem</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>o_que_evidencia</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>nome_original_arquivo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>capturado_em</t>
         </is>
@@ -476,7 +488,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>docs/img/01_setup</t>
+          <t>docs/img/base/01_setup</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -501,7 +513,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>02-carga_nb00_01_schemas.png</t>
+          <t>02-carga_nb01_01_schemas-volume.png</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -518,7 +530,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>docs/img/01_setup</t>
+          <t>docs/img/base/01_setup</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -543,7 +555,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>02-carga_nb00_02_landing-folders.png</t>
+          <t>02-carga_nb01_02_landing-folders.png</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -560,7 +572,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>docs/img/01_setup</t>
+          <t>docs/img/base/01_setup</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -602,7 +614,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -636,7 +648,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -670,7 +682,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -704,7 +716,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -738,7 +750,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -772,7 +784,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -806,7 +818,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -840,7 +852,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>docs/img/02_bronze_ingestion</t>
+          <t>docs/img/base/02_bronze_ingestion</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -874,7 +886,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -908,7 +920,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -942,7 +954,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -976,7 +988,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1010,7 +1022,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1044,7 +1056,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1078,7 +1090,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1112,7 +1124,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1146,7 +1158,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1180,7 +1192,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1214,7 +1226,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1248,7 +1260,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>docs/img/03_bronze_data_quality</t>
+          <t>docs/img/base/03_bronze_data_quality</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1273,6 +1285,48 @@
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>05-qualidade_ui_01_validacao-aneel-2022-2023.png</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>docs/img/complaints</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>05-qualidade</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>essencial</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Painel ANEEL de validacao das reclamacoes de 1o nivel (atualizado em 17/06/2025): diferencas acima de 10% entre 2022 e 2023 marcadas como indicio de erro, o que sustenta a exclusao de 2023 da serie</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>05-qualidade_ui_01_validacao-aneel-2022-2023.png</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>